<commit_message>
feat: Update fee notice structure and calculations
- Added new fields for serial number, O.M., robotic, and tuition in the fee notice.
- Updated sample data to reflect new fields and calculations.
- Enhanced fee total calculation to include new fields and handle total directly.
- Modified notice rendering to display new fields and updated layout.
- Improved PDF export functionality to accommodate new fee structure.
- Added a preview image for the pending fees notice.
- Included inspection data for the updated fee notice Excel template.
</commit_message>
<xml_diff>
--- a/public/Fee-Notice-Sample.xlsx
+++ b/public/Fee-Notice-Sample.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fee Notices" sheetId="1" r:id="Rba2d0cbc7b504560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fee Notices" sheetId="1" r:id="R506968e50af84cc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0;(#,##0);-"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -66,7 +67,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -90,11 +91,30 @@
     <x:xf numFmtId="200" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeeNotices" displayName="FeeNotices" ref="A1:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G6"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Student Name"/>
+    <x:tableColumn id="2" name="Father / Guardian"/>
+    <x:tableColumn id="3" name="ID No"/>
+    <x:tableColumn id="4" name="Class"/>
+    <x:tableColumn id="5" name="Fees"/>
+    <x:tableColumn id="6" name="Books"/>
+    <x:tableColumn id="7" name="Others"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -295,10 +315,10 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
@@ -319,17 +339,15 @@
         <x:v>Class</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>Old Balance</x:v>
+        <x:v>Fees</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>Fees</x:v>
+        <x:v>Books</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
-        <x:v>Books</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
         <x:v>Others</x:v>
       </x:c>
+      <x:c r="H1"/>
     </x:row>
     <x:row r="2" ht="20" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -344,18 +362,16 @@
       <x:c r="D2" s="9" t="str">
         <x:v>VI – A</x:v>
       </x:c>
-      <x:c r="E2" s="10" t="n">
-        <x:v>1200</x:v>
-      </x:c>
-      <x:c r="F2" s="10" t="n">
+      <x:c r="E2" s="11" t="n">
         <x:v>8000</x:v>
       </x:c>
-      <x:c r="G2" s="10" t="n">
+      <x:c r="F2" s="11" t="n">
         <x:v>1500</x:v>
       </x:c>
-      <x:c r="H2" s="10" t="n">
+      <x:c r="G2" s="11" t="n">
         <x:v>300</x:v>
       </x:c>
+      <x:c r="H2"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -370,18 +386,16 @@
       <x:c r="D3" s="9" t="str">
         <x:v>VI – B</x:v>
       </x:c>
-      <x:c r="E3" s="10" t="n">
+      <x:c r="E3" s="11" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="F3" s="11" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F3" s="10" t="n">
-        <x:v>8000</x:v>
-      </x:c>
-      <x:c r="G3" s="10" t="n">
-        <x:v>1200</x:v>
-      </x:c>
-      <x:c r="H3" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H3"/>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -396,18 +410,16 @@
       <x:c r="D4" s="9" t="str">
         <x:v>VII – A</x:v>
       </x:c>
-      <x:c r="E4" s="10" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="F4" s="10" t="n">
+      <x:c r="E4" s="11" t="n">
         <x:v>9200</x:v>
       </x:c>
-      <x:c r="G4" s="10" t="n">
+      <x:c r="F4" s="11" t="n">
         <x:v>1800</x:v>
       </x:c>
-      <x:c r="H4" s="10" t="n">
+      <x:c r="G4" s="11" t="n">
         <x:v>450</x:v>
       </x:c>
+      <x:c r="H4"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -422,18 +434,16 @@
       <x:c r="D5" s="9" t="str">
         <x:v>VII – B</x:v>
       </x:c>
-      <x:c r="E5" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="10" t="n">
+      <x:c r="E5" s="11" t="n">
         <x:v>9200</x:v>
       </x:c>
-      <x:c r="G5" s="10" t="n">
+      <x:c r="F5" s="11" t="n">
         <x:v>1500</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="n">
+      <x:c r="G5" s="11" t="n">
         <x:v>250</x:v>
       </x:c>
+      <x:c r="H5"/>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -448,20 +458,21 @@
       <x:c r="D6" s="9" t="str">
         <x:v>VIII – A</x:v>
       </x:c>
-      <x:c r="E6" s="10" t="n">
-        <x:v>2500</x:v>
-      </x:c>
-      <x:c r="F6" s="10" t="n">
+      <x:c r="E6" s="11" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="G6" s="10" t="n">
+      <x:c r="F6" s="11" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="H6" s="10" t="n">
+      <x:c r="G6" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="H6"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518819dc6d9d4576"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>